<commit_message>
site bien fonctionnel sauf MAJ factures fournisseurs
</commit_message>
<xml_diff>
--- a/plan_comptable_crediter.xlsx
+++ b/plan_comptable_crediter.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Desktop\projet-bd-fournisseurs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\a_mou\Desktop\Compta\compta_2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C87FD3-69B9-43F7-82AE-8288D1734E85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{5EAFE5E9-C3A5-496F-974B-3D12F3F3BAB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,11 +16,12 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
+  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="96">
   <si>
     <t>Numéro de compte</t>
   </si>
@@ -31,31 +32,283 @@
     <t>2000</t>
   </si>
   <si>
-    <t>Caisse</t>
-  </si>
-  <si>
     <t>2001</t>
   </si>
   <si>
-    <t>Banque</t>
-  </si>
-  <si>
-    <t>2002</t>
-  </si>
-  <si>
-    <t>Créances clients</t>
-  </si>
-  <si>
-    <t>2003</t>
-  </si>
-  <si>
-    <t>Dettes fournisseurs</t>
-  </si>
-  <si>
-    <t>2004</t>
-  </si>
-  <si>
-    <t>Stocks</t>
+    <t>1000</t>
+  </si>
+  <si>
+    <t>1001</t>
+  </si>
+  <si>
+    <t>1010</t>
+  </si>
+  <si>
+    <t>1011</t>
+  </si>
+  <si>
+    <t>1020</t>
+  </si>
+  <si>
+    <t>1021</t>
+  </si>
+  <si>
+    <t>1100</t>
+  </si>
+  <si>
+    <t>1101</t>
+  </si>
+  <si>
+    <t>1200</t>
+  </si>
+  <si>
+    <t>1201</t>
+  </si>
+  <si>
+    <t>1300</t>
+  </si>
+  <si>
+    <t>1301</t>
+  </si>
+  <si>
+    <t>1500</t>
+  </si>
+  <si>
+    <t>1501</t>
+  </si>
+  <si>
+    <t>1510</t>
+  </si>
+  <si>
+    <t>1511</t>
+  </si>
+  <si>
+    <t>1520</t>
+  </si>
+  <si>
+    <t>1521</t>
+  </si>
+  <si>
+    <t>2100</t>
+  </si>
+  <si>
+    <t>2101</t>
+  </si>
+  <si>
+    <t>2200</t>
+  </si>
+  <si>
+    <t>2201</t>
+  </si>
+  <si>
+    <t>2500</t>
+  </si>
+  <si>
+    <t>2501</t>
+  </si>
+  <si>
+    <t>2600</t>
+  </si>
+  <si>
+    <t>2601</t>
+  </si>
+  <si>
+    <t>2700</t>
+  </si>
+  <si>
+    <t>2701</t>
+  </si>
+  <si>
+    <t>2800</t>
+  </si>
+  <si>
+    <t>2801</t>
+  </si>
+  <si>
+    <t>2900</t>
+  </si>
+  <si>
+    <t>3000</t>
+  </si>
+  <si>
+    <t>3001</t>
+  </si>
+  <si>
+    <t>4000</t>
+  </si>
+  <si>
+    <t>4001</t>
+  </si>
+  <si>
+    <t>5000</t>
+  </si>
+  <si>
+    <t>5001</t>
+  </si>
+  <si>
+    <t>6000</t>
+  </si>
+  <si>
+    <t>6001</t>
+  </si>
+  <si>
+    <t>7000</t>
+  </si>
+  <si>
+    <t>7001</t>
+  </si>
+  <si>
+    <t>8000</t>
+  </si>
+  <si>
+    <t>8001</t>
+  </si>
+  <si>
+    <t>9000</t>
+  </si>
+  <si>
+    <t>9001</t>
+  </si>
+  <si>
+    <t>Caisse 1</t>
+  </si>
+  <si>
+    <t>Caisse 2</t>
+  </si>
+  <si>
+    <t>CCP 1</t>
+  </si>
+  <si>
+    <t>CCP 2</t>
+  </si>
+  <si>
+    <t>Banque 1</t>
+  </si>
+  <si>
+    <t>Banque 2</t>
+  </si>
+  <si>
+    <t>Débiteurs 1</t>
+  </si>
+  <si>
+    <t>Débiteurs 2</t>
+  </si>
+  <si>
+    <t>Stock 1</t>
+  </si>
+  <si>
+    <t>Stock2</t>
+  </si>
+  <si>
+    <t>Actif transitoire 1</t>
+  </si>
+  <si>
+    <t>Actif transitoire 2</t>
+  </si>
+  <si>
+    <t>Machine 1</t>
+  </si>
+  <si>
+    <t>Machine 2</t>
+  </si>
+  <si>
+    <t>Véhicule 1</t>
+  </si>
+  <si>
+    <t>Véhicule 2</t>
+  </si>
+  <si>
+    <t>Immeuble 1</t>
+  </si>
+  <si>
+    <t>Immeuble 2</t>
+  </si>
+  <si>
+    <t>Fournisseurs 1</t>
+  </si>
+  <si>
+    <t>Fournisseurs 2</t>
+  </si>
+  <si>
+    <t>Créancier 1</t>
+  </si>
+  <si>
+    <t>Créancier 2</t>
+  </si>
+  <si>
+    <t>Passif transitoire 1</t>
+  </si>
+  <si>
+    <t>Passif transitoire 2</t>
+  </si>
+  <si>
+    <t>Provision 1</t>
+  </si>
+  <si>
+    <t>Provision 2</t>
+  </si>
+  <si>
+    <t>Reserve 1</t>
+  </si>
+  <si>
+    <t>Reserve 2</t>
+  </si>
+  <si>
+    <t>Capital 1</t>
+  </si>
+  <si>
+    <t>Capital 2</t>
+  </si>
+  <si>
+    <t>Réserve légale 1</t>
+  </si>
+  <si>
+    <t>Réserve légale 2</t>
+  </si>
+  <si>
+    <t>Pertes et Profits reporté</t>
+  </si>
+  <si>
+    <t>Revenus 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Revenus 2</t>
+  </si>
+  <si>
+    <t>Achat 1</t>
+  </si>
+  <si>
+    <t>Achat 2</t>
+  </si>
+  <si>
+    <t>Salaire 1</t>
+  </si>
+  <si>
+    <t>Salaire 2</t>
+  </si>
+  <si>
+    <t>Frais d'exploitation 1</t>
+  </si>
+  <si>
+    <t>Frais d'exploitation 2</t>
+  </si>
+  <si>
+    <t>Intérêts 1</t>
+  </si>
+  <si>
+    <t>Intérêts 2</t>
+  </si>
+  <si>
+    <t>Divers 1</t>
+  </si>
+  <si>
+    <t>Divers 2</t>
+  </si>
+  <si>
+    <t>Compte de résultat 1</t>
+  </si>
+  <si>
+    <t>Compte de résultat 2</t>
   </si>
 </sst>
 </file>
@@ -84,15 +337,27 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
+        <bgColor theme="4" tint="0.59999389629810485"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor theme="4" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -115,16 +380,74 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom style="thin">
+        <color theme="0"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color theme="0"/>
+      </left>
+      <right style="thin">
+        <color theme="0"/>
+      </right>
+      <top style="thin">
+        <color theme="0"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -427,7 +750,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="23.5546875" customWidth="1"/>
@@ -444,49 +767,385 @@
       <c r="C1" s="2"/>
     </row>
     <row r="2" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+      <c r="A3" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="2"/>
+    </row>
+    <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+      <c r="A4" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="2"/>
+    </row>
+    <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+      <c r="A5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="C5" s="2"/>
+    </row>
+    <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.35">
+      <c r="A6" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C6" s="2"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B15" s="7" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" s="7" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A18" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A20" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B20" s="6" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A3" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" s="2"/>
-    </row>
-    <row r="4" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A4" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="2"/>
-    </row>
-    <row r="5" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A5" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" s="2"/>
-    </row>
-    <row r="6" spans="1:3" ht="18" x14ac:dyDescent="0.35">
-      <c r="A6" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="2"/>
+      <c r="B21" s="7" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A22" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A24" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" s="7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A26" s="3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B27" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A28" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B28" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="B29" s="7" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A30" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B30" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B31" s="7" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A32" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B32" s="6" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="B33" s="7" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B34" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B35" s="7" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A36" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B36" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B37" s="7" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A38" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B38" s="6" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B39" s="7" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B41" s="7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="B43" s="7" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B45" s="7" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="B46" s="6" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B47" s="7" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B48" s="8" t="s">
+        <v>95</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>